<commit_message>
add: cases for the rules no fixture caught
Four rules held only by the code. Each is now pinned by the book that
owns the subject:

formulas -- a relative reference above or below the band keeps the
distance it had after room was made, as Excel's Insert Copied Cells
does, rather than being fixed in place.

follow -- a conditional format and a validation lying inside the band
repeat once per copy; a defined name reaching over it stretches by the
rows inserted, and no further.

values -- a trailing full-width space, which needs xml:space="preserve"
on a text that a leading or trailing ASCII space would not distinguish.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/data_golden/follow.expected.xlsx
+++ b/tests/data_golden/follow.expected.xlsx
@@ -31,6 +31,8 @@
     <sheet name="follow-rc-merged" sheetId="22" r:id="rId25"/>
     <sheet name="follow-cr-merged" sheetId="23" r:id="rId26"/>
     <sheet name="follow-cc-merged" sheetId="24" r:id="rId27"/>
+    <sheet name="follow-r-cond-format-inside" sheetId="25" r:id="rId28"/>
+    <sheet name="follow-r-defined-name-inside" sheetId="26" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="FolRName">'follow-r-defined-name'!$B$3:$E$5</definedName>
@@ -39,13 +41,14 @@
     <definedName localSheetId="7" name="_xlnm.Print_Area">'follow-c-print-area'!$B$2:$G$4</definedName>
     <definedName hidden="true" localSheetId="8" name="_xlnm._FilterDatabase">'follow-r-filter'!$B$2:$E$5</definedName>
     <definedName hidden="true" localSheetId="9" name="_xlnm._FilterDatabase">'follow-c-filter'!$B$2:$E$3</definedName>
+    <definedName name="FolRInside">'follow-r-defined-name-inside'!$B$2:$C$3</definedName>
   </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="53">
   <si>
     <t>Name</t>
   </si>
@@ -182,19 +185,19 @@
     <t>Sales</t>
   </si>
   <si>
-    <t>No. 1</t>
-  </si>
-  <si>
-    <t>No. 2</t>
-  </si>
-  <si>
-    <t>Sales total</t>
+    <t xml:space="preserve">No. 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sales total</t>
   </si>
   <si>
     <t>Dev</t>
   </si>
   <si>
-    <t>Dev total</t>
+    <t xml:space="preserve">Dev total</t>
   </si>
   <si>
     <t>A</t>
@@ -244,11 +247,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -315,32 +325,32 @@
     </xdr:sp>
     <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Shape 3" descr=""/>
-        <xdr:cNvSpPr txBox="true"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+  <twoCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>2</col>
+      <colOff>38100</colOff>
+      <row>5</row>
+      <rowOff>95250</rowOff>
+    </to>
+    <sp macro="" textlink="">
+      <nvSpPr>
+        <cNvPr id="3" name="Shape 3" descr=""/>
+        <cNvSpPr txBox="true"/>
+      </nvSpPr>
+      <spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="952500" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-      <xdr:style>
+      </spPr>
+      <style>
         <a:lnRef idx="0">
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
@@ -353,8 +363,8 @@
         <a:fontRef idx="minor">
           <a:schemeClr val="tx1"/>
         </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
+      </style>
+      <txBody>
         <a:bodyPr anchor="t" anchorCtr="false" rot="0" horzOverflow="clip" spcFirstLastPara="false" vertOverflow="clip" wrap="none"/>
         <a:p>
           <a:r>
@@ -367,36 +377,36 @@
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="Shape 4" descr=""/>
-        <xdr:cNvSpPr txBox="true"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+      </txBody>
+    </sp>
+    <clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </twoCellAnchor>
+  <twoCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>2</col>
+      <colOff>38100</colOff>
+      <row>6</row>
+      <rowOff>95250</rowOff>
+    </to>
+    <sp macro="" textlink="">
+      <nvSpPr>
+        <cNvPr id="4" name="Shape 4" descr=""/>
+        <cNvSpPr txBox="true"/>
+      </nvSpPr>
+      <spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="952500" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-      <xdr:style>
+      </spPr>
+      <style>
         <a:lnRef idx="0">
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
@@ -409,8 +419,8 @@
         <a:fontRef idx="minor">
           <a:schemeClr val="tx1"/>
         </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
+      </style>
+      <txBody>
         <a:bodyPr anchor="t" anchorCtr="false" rot="0" horzOverflow="clip" spcFirstLastPara="false" vertOverflow="clip" wrap="none"/>
         <a:p>
           <a:r>
@@ -423,10 +433,10 @@
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
+      </txBody>
+    </sp>
+    <clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -488,32 +498,32 @@
     </xdr:sp>
     <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Shape 3" descr=""/>
-        <xdr:cNvSpPr txBox="true"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+  <twoCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>4</col>
+      <colOff>38100</colOff>
+      <row>3</row>
+      <rowOff>95250</rowOff>
+    </to>
+    <sp macro="" textlink="">
+      <nvSpPr>
+        <cNvPr id="3" name="Shape 3" descr=""/>
+        <cNvSpPr txBox="true"/>
+      </nvSpPr>
+      <spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="952500" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-      <xdr:style>
+      </spPr>
+      <style>
         <a:lnRef idx="0">
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
@@ -526,8 +536,8 @@
         <a:fontRef idx="minor">
           <a:schemeClr val="tx1"/>
         </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
+      </style>
+      <txBody>
         <a:bodyPr anchor="t" anchorCtr="false" rot="0" horzOverflow="clip" spcFirstLastPara="false" vertOverflow="clip" wrap="none"/>
         <a:p>
           <a:r>
@@ -540,36 +550,36 @@
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="Shape 4" descr=""/>
-        <xdr:cNvSpPr txBox="true"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+      </txBody>
+    </sp>
+    <clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </twoCellAnchor>
+  <twoCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>5</col>
+      <colOff>38100</colOff>
+      <row>3</row>
+      <rowOff>95250</rowOff>
+    </to>
+    <sp macro="" textlink="">
+      <nvSpPr>
+        <cNvPr id="4" name="Shape 4" descr=""/>
+        <cNvSpPr txBox="true"/>
+      </nvSpPr>
+      <spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="952500" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-      <xdr:style>
+      </spPr>
+      <style>
         <a:lnRef idx="0">
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
@@ -582,8 +592,8 @@
         <a:fontRef idx="minor">
           <a:schemeClr val="tx1"/>
         </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
+      </style>
+      <txBody>
         <a:bodyPr anchor="t" anchorCtr="false" rot="0" horzOverflow="clip" spcFirstLastPara="false" vertOverflow="clip" wrap="none"/>
         <a:p>
           <a:r>
@@ -596,10 +606,10 @@
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
+      </txBody>
+    </sp>
+    <clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -661,32 +671,32 @@
     </xdr:sp>
     <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Shape 3" descr=""/>
-        <xdr:cNvSpPr txBox="true"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+  <twoCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>3</col>
+      <colOff>38100</colOff>
+      <row>5</row>
+      <rowOff>95250</rowOff>
+    </to>
+    <sp macro="" textlink="">
+      <nvSpPr>
+        <cNvPr id="3" name="Shape 3" descr=""/>
+        <cNvSpPr txBox="true"/>
+      </nvSpPr>
+      <spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="952500" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-      <xdr:style>
+      </spPr>
+      <style>
         <a:lnRef idx="0">
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
@@ -699,8 +709,8 @@
         <a:fontRef idx="minor">
           <a:schemeClr val="tx1"/>
         </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
+      </style>
+      <txBody>
         <a:bodyPr anchor="t" anchorCtr="false" rot="0" horzOverflow="clip" spcFirstLastPara="false" vertOverflow="clip" wrap="none"/>
         <a:p>
           <a:r>
@@ -713,36 +723,36 @@
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="Shape 4" descr=""/>
-        <xdr:cNvSpPr txBox="true"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+      </txBody>
+    </sp>
+    <clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </twoCellAnchor>
+  <twoCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>3</col>
+      <colOff>38100</colOff>
+      <row>8</row>
+      <rowOff>95250</rowOff>
+    </to>
+    <sp macro="" textlink="">
+      <nvSpPr>
+        <cNvPr id="4" name="Shape 4" descr=""/>
+        <cNvSpPr txBox="true"/>
+      </nvSpPr>
+      <spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="952500" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-      <xdr:style>
+      </spPr>
+      <style>
         <a:lnRef idx="0">
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
@@ -755,8 +765,8 @@
         <a:fontRef idx="minor">
           <a:schemeClr val="tx1"/>
         </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
+      </style>
+      <txBody>
         <a:bodyPr anchor="t" anchorCtr="false" rot="0" horzOverflow="clip" spcFirstLastPara="false" vertOverflow="clip" wrap="none"/>
         <a:p>
           <a:r>
@@ -769,10 +779,10 @@
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
+      </txBody>
+    </sp>
+    <clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -834,32 +844,32 @@
     </xdr:sp>
     <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Shape 3" descr=""/>
-        <xdr:cNvSpPr txBox="true"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+  <twoCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>4</col>
+      <colOff>38100</colOff>
+      <row>4</row>
+      <rowOff>95250</rowOff>
+    </to>
+    <sp macro="" textlink="">
+      <nvSpPr>
+        <cNvPr id="3" name="Shape 3" descr=""/>
+        <cNvSpPr txBox="true"/>
+      </nvSpPr>
+      <spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="952500" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-      <xdr:style>
+      </spPr>
+      <style>
         <a:lnRef idx="0">
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
@@ -872,8 +882,8 @@
         <a:fontRef idx="minor">
           <a:schemeClr val="tx1"/>
         </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
+      </style>
+      <txBody>
         <a:bodyPr anchor="t" anchorCtr="false" rot="0" horzOverflow="clip" spcFirstLastPara="false" vertOverflow="clip" wrap="none"/>
         <a:p>
           <a:r>
@@ -886,36 +896,36 @@
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="Shape 4" descr=""/>
-        <xdr:cNvSpPr txBox="true"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+      </txBody>
+    </sp>
+    <clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </twoCellAnchor>
+  <twoCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>3</col>
+      <colOff>38100</colOff>
+      <row>6</row>
+      <rowOff>95250</rowOff>
+    </to>
+    <sp macro="" textlink="">
+      <nvSpPr>
+        <cNvPr id="4" name="Shape 4" descr=""/>
+        <cNvSpPr txBox="true"/>
+      </nvSpPr>
+      <spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="952500" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-      <xdr:style>
+      </spPr>
+      <style>
         <a:lnRef idx="0">
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
@@ -928,8 +938,8 @@
         <a:fontRef idx="minor">
           <a:schemeClr val="tx1"/>
         </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
+      </style>
+      <txBody>
         <a:bodyPr anchor="t" anchorCtr="false" rot="0" horzOverflow="clip" spcFirstLastPara="false" vertOverflow="clip" wrap="none"/>
         <a:p>
           <a:r>
@@ -942,36 +952,36 @@
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="Shape 5" descr=""/>
-        <xdr:cNvSpPr txBox="true"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+      </txBody>
+    </sp>
+    <clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </twoCellAnchor>
+  <twoCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>4</col>
+      <colOff>38100</colOff>
+      <row>6</row>
+      <rowOff>95250</rowOff>
+    </to>
+    <sp macro="" textlink="">
+      <nvSpPr>
+        <cNvPr id="5" name="Shape 5" descr=""/>
+        <cNvSpPr txBox="true"/>
+      </nvSpPr>
+      <spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="952500" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-      <xdr:style>
+      </spPr>
+      <style>
         <a:lnRef idx="0">
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
@@ -984,8 +994,8 @@
         <a:fontRef idx="minor">
           <a:schemeClr val="tx1"/>
         </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
+      </style>
+      <txBody>
         <a:bodyPr anchor="t" anchorCtr="false" rot="0" horzOverflow="clip" spcFirstLastPara="false" vertOverflow="clip" wrap="none"/>
         <a:p>
           <a:r>
@@ -998,10 +1008,10 @@
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
+      </txBody>
+    </sp>
+    <clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1063,32 +1073,32 @@
     </xdr:sp>
     <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Shape 3" descr=""/>
-        <xdr:cNvSpPr txBox="true"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+  <twoCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>2</col>
+      <colOff>38100</colOff>
+      <row>5</row>
+      <rowOff>95250</rowOff>
+    </to>
+    <sp macro="" textlink="">
+      <nvSpPr>
+        <cNvPr id="3" name="Shape 3" descr=""/>
+        <cNvSpPr txBox="true"/>
+      </nvSpPr>
+      <spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="952500" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-      <xdr:style>
+      </spPr>
+      <style>
         <a:lnRef idx="0">
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
@@ -1101,8 +1111,8 @@
         <a:fontRef idx="minor">
           <a:schemeClr val="tx1"/>
         </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
+      </style>
+      <txBody>
         <a:bodyPr anchor="t" anchorCtr="false" rot="0" horzOverflow="clip" spcFirstLastPara="false" vertOverflow="clip" wrap="none"/>
         <a:p>
           <a:r>
@@ -1115,36 +1125,36 @@
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="Shape 4" descr=""/>
-        <xdr:cNvSpPr txBox="true"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+      </txBody>
+    </sp>
+    <clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </twoCellAnchor>
+  <twoCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>3</col>
+      <colOff>38100</colOff>
+      <row>4</row>
+      <rowOff>95250</rowOff>
+    </to>
+    <sp macro="" textlink="">
+      <nvSpPr>
+        <cNvPr id="4" name="Shape 4" descr=""/>
+        <cNvSpPr txBox="true"/>
+      </nvSpPr>
+      <spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="952500" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-      <xdr:style>
+      </spPr>
+      <style>
         <a:lnRef idx="0">
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
@@ -1157,8 +1167,8 @@
         <a:fontRef idx="minor">
           <a:schemeClr val="tx1"/>
         </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
+      </style>
+      <txBody>
         <a:bodyPr anchor="t" anchorCtr="false" rot="0" horzOverflow="clip" spcFirstLastPara="false" vertOverflow="clip" wrap="none"/>
         <a:p>
           <a:r>
@@ -1171,36 +1181,36 @@
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="Shape 5" descr=""/>
-        <xdr:cNvSpPr txBox="true"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+      </txBody>
+    </sp>
+    <clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </twoCellAnchor>
+  <twoCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>3</col>
+      <colOff>38100</colOff>
+      <row>5</row>
+      <rowOff>95250</rowOff>
+    </to>
+    <sp macro="" textlink="">
+      <nvSpPr>
+        <cNvPr id="5" name="Shape 5" descr=""/>
+        <cNvSpPr txBox="true"/>
+      </nvSpPr>
+      <spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="952500" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-      <xdr:style>
+      </spPr>
+      <style>
         <a:lnRef idx="0">
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
@@ -1213,8 +1223,8 @@
         <a:fontRef idx="minor">
           <a:schemeClr val="tx1"/>
         </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
+      </style>
+      <txBody>
         <a:bodyPr anchor="t" anchorCtr="false" rot="0" horzOverflow="clip" spcFirstLastPara="false" vertOverflow="clip" wrap="none"/>
         <a:p>
           <a:r>
@@ -1227,10 +1237,10 @@
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
+      </txBody>
+    </sp>
+    <clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1292,32 +1302,32 @@
     </xdr:sp>
     <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Shape 3" descr=""/>
-        <xdr:cNvSpPr txBox="true"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+  <twoCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>4</col>
+      <colOff>38100</colOff>
+      <row>4</row>
+      <rowOff>95250</rowOff>
+    </to>
+    <sp macro="" textlink="">
+      <nvSpPr>
+        <cNvPr id="3" name="Shape 3" descr=""/>
+        <cNvSpPr txBox="true"/>
+      </nvSpPr>
+      <spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="952500" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-      <xdr:style>
+      </spPr>
+      <style>
         <a:lnRef idx="0">
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
@@ -1330,8 +1340,8 @@
         <a:fontRef idx="minor">
           <a:schemeClr val="tx1"/>
         </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
+      </style>
+      <txBody>
         <a:bodyPr anchor="t" anchorCtr="false" rot="0" horzOverflow="clip" spcFirstLastPara="false" vertOverflow="clip" wrap="none"/>
         <a:p>
           <a:r>
@@ -1344,36 +1354,36 @@
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="Shape 4" descr=""/>
-        <xdr:cNvSpPr txBox="true"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+      </txBody>
+    </sp>
+    <clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </twoCellAnchor>
+  <twoCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>7</col>
+      <colOff>38100</colOff>
+      <row>4</row>
+      <rowOff>95250</rowOff>
+    </to>
+    <sp macro="" textlink="">
+      <nvSpPr>
+        <cNvPr id="4" name="Shape 4" descr=""/>
+        <cNvSpPr txBox="true"/>
+      </nvSpPr>
+      <spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="952500" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-      <xdr:style>
+      </spPr>
+      <style>
         <a:lnRef idx="0">
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
@@ -1386,8 +1396,8 @@
         <a:fontRef idx="minor">
           <a:schemeClr val="tx1"/>
         </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
+      </style>
+      <txBody>
         <a:bodyPr anchor="t" anchorCtr="false" rot="0" horzOverflow="clip" spcFirstLastPara="false" vertOverflow="clip" wrap="none"/>
         <a:p>
           <a:r>
@@ -1400,10 +1410,10 @@
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
+      </txBody>
+    </sp>
+    <clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2655,6 +2665,120 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
+    <col customWidth="true" max="1" min="1" width="3"/>
+    <col customWidth="true" max="5" min="2" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8">
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B3:C3 B5:C5 B7:C7">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" operator="between" sqref="B4 B6 B8" type="textLength">
+      <formula1>1</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
+  </dataValidations>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
+    <col customWidth="true" max="1" min="1" width="3"/>
+    <col customWidth="true" max="5" min="2" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>

</xml_diff>